<commit_message>
Add campaign source divergence tracking
</commit_message>
<xml_diff>
--- a/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
+++ b/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
@@ -18,17 +18,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core_vs_Pack" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUN_Assets" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peso_Assets" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist_Teste" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens_Campanha" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC_Mecanicas" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Fases" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faccoes" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mundo_Biomas" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteudo_Futuro" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divergencias" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core_vs_Pack" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUN_Assets" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peso_Assets" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist_Teste" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens_Campanha" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC_Mecanicas" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Fases" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faccoes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mundo_Biomas" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteudo_Futuro" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -347,8 +348,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="PainelFocoTable" displayName="PainelFocoTable" ref="A17:D22" headerRowCount="1">
-  <autoFilter ref="A17:D22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="PainelFocoTable" displayName="PainelFocoTable" ref="A17:D23" headerRowCount="1">
+  <autoFilter ref="A17:D23"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Sinal"/>
     <tableColumn id="2" name="Objetivo"/>
@@ -386,7 +387,25 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="CorePackTable" displayName="CorePackTable" ref="A4:F12" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="DivergenciasTable" displayName="DivergenciasTable" ref="A4:I11" headerRowCount="1">
+  <autoFilter ref="A4:I11"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Status"/>
+    <tableColumn id="2" name="Tipo"/>
+    <tableColumn id="3" name="Personagem"/>
+    <tableColumn id="4" name="Nome no app"/>
+    <tableColumn id="5" name="Nome/pasta lore"/>
+    <tableColumn id="6" name="Faccao/Pasta"/>
+    <tableColumn id="7" name="Detalhe"/>
+    <tableColumn id="8" name="Acao sugerida"/>
+    <tableColumn id="9" name="Fonte"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CorePackTable" displayName="CorePackTable" ref="A4:F12" headerRowCount="1">
   <autoFilter ref="A4:F12"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Bloco"/>
@@ -400,8 +419,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="MunAssetsTable" displayName="MunAssetsTable" ref="A4:J127" headerRowCount="1">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="MunAssetsTable" displayName="MunAssetsTable" ref="A4:J127" headerRowCount="1">
   <autoFilter ref="A4:J127"/>
   <tableColumns count="10">
     <tableColumn id="1" name="ID"/>
@@ -419,8 +438,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="HeavyOriginalsTable" displayName="HeavyOriginalsTable" ref="A4:G84" headerRowCount="1">
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="HeavyOriginalsTable" displayName="HeavyOriginalsTable" ref="A4:G84" headerRowCount="1">
   <autoFilter ref="A4:G84"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Original"/>
@@ -435,8 +454,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="ChecklistTable" displayName="ChecklistTable" ref="A4:F14" headerRowCount="1">
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="ChecklistTable" displayName="ChecklistTable" ref="A4:F14" headerRowCount="1">
   <autoFilter ref="A4:F14"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Prioridade"/>
@@ -450,8 +469,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="CampaignCharactersTable" displayName="CampaignCharactersTable" ref="A4:L55" headerRowCount="1">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="CampaignCharactersTable" displayName="CampaignCharactersTable" ref="A4:L55" headerRowCount="1">
   <autoFilter ref="A4:L55"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Status"/>
@@ -471,8 +490,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="NpcMechanicsTable" displayName="NpcMechanicsTable" ref="A4:X55" headerRowCount="1">
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="NpcMechanicsTable" displayName="NpcMechanicsTable" ref="A4:X55" headerRowCount="1">
   <autoFilter ref="A4:X55"/>
   <tableColumns count="24">
     <tableColumn id="1" name="Status"/>
@@ -504,8 +523,18 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="ProtagonistasTable" displayName="ProtagonistasTable" ref="A4:O11" headerRowCount="1">
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ControleRegrasTable" displayName="ControleRegrasTable" ref="G13:G18" headerRowCount="1">
+  <autoFilter ref="G13:G18"/>
+  <tableColumns count="1">
+    <tableColumn id="7" name="Regra"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="ProtagonistasTable" displayName="ProtagonistasTable" ref="A4:O11" headerRowCount="1">
   <autoFilter ref="A4:O11"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Status"/>
@@ -528,18 +557,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ControleRegrasTable" displayName="ControleRegrasTable" ref="G13:G18" headerRowCount="1">
-  <autoFilter ref="G13:G18"/>
-  <tableColumns count="1">
-    <tableColumn id="7" name="Regra"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="BossesFasesTable" displayName="BossesFasesTable" ref="A4:O19" headerRowCount="1">
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="BossesFasesTable" displayName="BossesFasesTable" ref="A4:O19" headerRowCount="1">
   <autoFilter ref="A4:O19"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Status"/>
@@ -562,8 +581,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="FaccoesTable" displayName="FaccoesTable" ref="A4:M10" headerRowCount="1">
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="FaccoesTable" displayName="FaccoesTable" ref="A4:M10" headerRowCount="1">
   <autoFilter ref="A4:M10"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Status"/>
@@ -584,8 +603,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="MundoBiomasTable" displayName="MundoBiomasTable" ref="A4:N12" headerRowCount="1">
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="MundoBiomasTable" displayName="MundoBiomasTable" ref="A4:N12" headerRowCount="1">
   <autoFilter ref="A4:N12"/>
   <tableColumns count="14">
     <tableColumn id="1" name="Status"/>
@@ -607,8 +626,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="FutureContentTable" displayName="FutureContentTable" ref="A4:G10" headerRowCount="1">
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="FutureContentTable" displayName="FutureContentTable" ref="A4:G10" headerRowCount="1">
   <autoFilter ref="A4:G10"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Sistema"/>
@@ -2048,6 +2067,424 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="61" customWidth="1" min="7" max="7"/>
+    <col width="61" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Divergencias De Fonte App x Lore</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="19" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Use esta aba para resolver confusoes de nome, pasta, arquivo vazio e lore que ainda nao entrou no app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Personagem</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Nome no app</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Nome/pasta lore</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Faccao/Pasta</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Detalhe</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Acao sugerida</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Nome divergente</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Sélian Velan</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Sélian Velan</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Sélian</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Vila do Conhecimento Absorvido</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Vinculo aceito por nome parcial; conferir se e apelido/erro de grafia intencional.</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Padronizar nome no app ou registrar alias aprovado para nao confundir com outro NPC.</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>(D) Villa (Planicie) (Protagonistas)/Sélian (Protagonista Kairos ; Kuster)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Lore reconstruida do app</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Yor</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Yor</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Yor</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Ordem do Véu Cinza</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>A ficha foi reconstruida a partir do workspace do app, nao de um arquivo original antigo.</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Revisar com o mestre quando houver tempo e decidir se vira fonte definitiva.</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>(C) Detetives (Véu cinzento)(.)/Yor (Yor Spy family)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Nome divergente</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Liryssa</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Liryssa</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Lyrissa</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Companhia da Maré Livre</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Vinculo aceito por alias nome; conferir se e apelido/erro de grafia intencional.</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Padronizar nome no app ou registrar alias aprovado para nao confundir com outro NPC.</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>(E) Aventureiros Maré (Mar)/Lyrissa (Capitã)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Lore reconstruida do app</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Varden</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Varden</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Varden</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Companhia da Maré Livre</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>A ficha foi reconstruida a partir do workspace do app, nao de um arquivo original antigo.</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Revisar com o mestre quando houver tempo e decidir se vira fonte definitiva.</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>(E) Aventureiros Maré (Mar)/Varden (Frankstain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Lore reconstruida do app</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Bront</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Bront</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Bront</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Companhia da Maré Livre</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>A ficha foi reconstruida a partir do workspace do app, nao de um arquivo original antigo.</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Revisar com o mestre quando houver tempo e decidir se vira fonte definitiva.</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>(E) Aventureiros Maré (Mar)/Bront (Cozinheiro Naval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Nome divergente</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Maira Velan</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Maira Velan</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Maira</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Vila do Conhecimento Absorvido</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Vinculo aceito por nome parcial; conferir se e apelido/erro de grafia intencional.</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Padronizar nome no app ou registrar alias aprovado para nao confundir com outro NPC.</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>(D) Villa (Planicie) (Protagonistas)/Maira (Mãe de Sélian)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CRITICO</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>APP sem pasta lore</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Teste</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Teste</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Ordem do Vazio Sereno</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Personagem existe no app, mas nenhuma pasta/arquivo de lore foi vinculado.</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Criar/vincular pasta em 01_LORE ou marcar conscientemente como somente-app.</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>C:\Users\danie\AppData\Roaming\FUSHI\workspace.json</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2373,7 +2810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8868,7 +9305,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11429,7 +11866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11824,7 +12261,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15081,7 +15518,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20580,7 +21017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21177,1140 +21614,6 @@
       <c r="O11" s="8" t="inlineStr">
         <is>
           <t>character-dc758c81-53f2-4cea-953e-ee205f8586a2</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
-    <col width="51" customWidth="1" min="15" max="15"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Bosses, Cataclisma E Fichas Avancadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="19" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Planejamento de entidades com fases, mapas, aparencias, VFX/3D, interludios e controle de estado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Personagem</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Classe ficha</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Faccao</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Local</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Historia app</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Lore arquivo</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Eventos</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Fases</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Mapas</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Img</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>Dominio/VFX</t>
-        </is>
-      </c>
-      <c r="N4" s="6" t="inlineStr">
-        <is>
-          <t>Controle necessario</t>
-        </is>
-      </c>
-      <c r="O4" s="6" t="inlineStr">
-        <is>
-          <t>Lore path</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Yanzik</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>FUSHI Escuro</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Viajante</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O5" s="8" t="inlineStr">
-        <is>
-          <t>(B) FUSHI escuro (Andarilho)(.)/Yanzik (Guts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Seraph</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>FUSHI Escuro</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Andarilho</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N6" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O6" s="8" t="inlineStr">
-        <is>
-          <t>(B) FUSHI escuro (Andarilho)(.)/Seraph (Griffith)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Ryoku</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>FUSHI Escuro</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Ruinas</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="J7" s="8" t="n">
-        <v>107</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N7" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O7" s="8" t="inlineStr">
-        <is>
-          <t>(B) FUSHI escuro (Andarilho)(.)/Ryoku (Sukuna)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Maelra</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Companhia da Maré Livre</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Praia</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N8" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O8" s="8" t="inlineStr">
-        <is>
-          <t>(E) Aventureiros Maré (Mar)/Maelra (Cura)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Veyra</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Companhia da Maré Livre</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Praia</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N9" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O9" s="8" t="inlineStr">
-        <is>
-          <t>(E) Aventureiros Maré (Mar)/Veyra (Yumeko)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - ficha avancada</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Nyx</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>FICHA AVANCADA / BOSS</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Companhia da Maré Livre</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Litoral</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N10" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
-        </is>
-      </c>
-      <c r="O10" s="8" t="inlineStr">
-        <is>
-          <t>(E) Aventureiros Maré (Mar)/Nyx (Cyber Punk Gamer)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - ficha avancada</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Morghast</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>FICHA AVANCADA / BOSS</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Vulcão</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="J11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Morghast (Guardião 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - ficha avancada</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Euryaleth</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>FICHA AVANCADA / BOSS</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Vulcão</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="10" t="inlineStr">
-        <is>
-          <t>nao detectado</t>
-        </is>
-      </c>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
-        </is>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Euryaleth (Guardião 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - ficha avancada</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Vorashk</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>FICHA AVANCADA / BOSS</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Vulcão</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="10" t="inlineStr">
-        <is>
-          <t>nao detectado</t>
-        </is>
-      </c>
-      <c r="N13" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Vorashk (Guardião 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - ficha avancada</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Aeronyx</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>FICHA AVANCADA / BOSS</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Vulcão</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="J14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N14" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Aeronyx (Guardião 4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - ficha avancada</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Thal’Zhyr</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>FICHA AVANCADA / BOSS</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Oceano</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="10" t="inlineStr">
-        <is>
-          <t>nao detectado</t>
-        </is>
-      </c>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Thal’Zhyr (Guardião 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Astrael</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Nucleo Paradoxial</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="8" t="n">
-        <v>23</v>
-      </c>
-      <c r="J16" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="10" t="inlineStr">
-        <is>
-          <t>nao detectado</t>
-        </is>
-      </c>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O16" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Astrael (Guardião 6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Orian</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Vila do Conhecimento Absorvido</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Vila Inicial</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>39</v>
-      </c>
-      <c r="K17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="10" t="inlineStr">
-        <is>
-          <t>nao detectado</t>
-        </is>
-      </c>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O17" s="8" t="inlineStr">
-        <is>
-          <t>(D) Villa (Planicie) (Protagonistas)/Orian (Marido Cartografo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Kazuo</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Vila do Conhecimento Absorvido</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Vila Inicial</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="10" t="inlineStr">
-        <is>
-          <t>nao detectado</t>
-        </is>
-      </c>
-      <c r="N18" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O18" s="8" t="inlineStr">
-        <is>
-          <t>(D) Villa (Planicie) (Protagonistas)/Kazuo (Mestre de Renji)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>FOCO - boss cataclisma</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Vhazaryon</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>BOSS CATACLISMA</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Guardiões do Vulcão</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Vulcão Selado</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>falta</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="8" t="n">
-        <v>61</v>
-      </c>
-      <c r="J19" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="K19" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="L19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>requer VFX</t>
-        </is>
-      </c>
-      <c r="N19" s="8" t="inlineStr">
-        <is>
-          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
-        </is>
-      </c>
-      <c r="O19" s="8" t="inlineStr">
-        <is>
-          <t>(F) Guardiões (Vulcão)/Vhazaryon (Dragão FUSHI)</t>
         </is>
       </c>
     </row>
@@ -22695,6 +21998,1140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="51" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bosses, Cataclisma E Fichas Avancadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="19" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Planejamento de entidades com fases, mapas, aparencias, VFX/3D, interludios e controle de estado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Personagem</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Classe ficha</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Faccao</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Historia app</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Lore arquivo</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Eventos</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Fases</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Mapas</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>Img</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>Dominio/VFX</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>Controle necessario</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>Lore path</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Yanzik</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>FUSHI Escuro</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Viajante</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>(B) FUSHI escuro (Andarilho)(.)/Yanzik (Guts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Seraph</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>FUSHI Escuro</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Andarilho</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>(B) FUSHI escuro (Andarilho)(.)/Seraph (Griffith)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Ryoku</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>FUSHI Escuro</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Ruinas</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>107</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>(B) FUSHI escuro (Andarilho)(.)/Ryoku (Sukuna)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Maelra</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Companhia da Maré Livre</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Praia</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>(E) Aventureiros Maré (Mar)/Maelra (Cura)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Veyra</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Companhia da Maré Livre</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Praia</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>(E) Aventureiros Maré (Mar)/Veyra (Yumeko)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - ficha avancada</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Nyx</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>FICHA AVANCADA / BOSS</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Companhia da Maré Livre</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Litoral</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>(E) Aventureiros Maré (Mar)/Nyx (Cyber Punk Gamer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - ficha avancada</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Morghast</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>FICHA AVANCADA / BOSS</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Vulcão</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Morghast (Guardião 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - ficha avancada</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Euryaleth</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>FICHA AVANCADA / BOSS</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Vulcão</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>nao detectado</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Euryaleth (Guardião 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - ficha avancada</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Vorashk</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>FICHA AVANCADA / BOSS</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Vulcão</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="10" t="inlineStr">
+        <is>
+          <t>nao detectado</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Vorashk (Guardião 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - ficha avancada</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Aeronyx</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>FICHA AVANCADA / BOSS</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Vulcão</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Aeronyx (Guardião 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - ficha avancada</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Thal’Zhyr</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>FICHA AVANCADA / BOSS</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Oceano</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="10" t="inlineStr">
+        <is>
+          <t>nao detectado</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com mecanicas especiais, imagem/lore e interludio.</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Thal’Zhyr (Guardião 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Astrael</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Nucleo Paradoxial</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t>nao detectado</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Astrael (Guardião 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Orian</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Vila do Conhecimento Absorvido</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Vila Inicial</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="10" t="inlineStr">
+        <is>
+          <t>nao detectado</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>(D) Villa (Planicie) (Protagonistas)/Orian (Marido Cartografo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Kazuo</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Vila do Conhecimento Absorvido</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Vila Inicial</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="10" t="inlineStr">
+        <is>
+          <t>nao detectado</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>(D) Villa (Planicie) (Protagonistas)/Kazuo (Mestre de Renji)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>FOCO - boss cataclisma</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Vhazaryon</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>BOSS CATACLISMA</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Guardiões do Vulcão</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Vulcão Selado</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>falta</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="J19" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
+        <is>
+          <t>requer VFX</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>Ficha avancada com fases, mapas, aparencias, VFX/3D, interludios e estado de fase.</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
+          <t>(F) Guardiões (Vulcão)/Vhazaryon (Dragão FUSHI)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -23124,7 +23561,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23691,7 +24128,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29329,7 +29766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -29484,7 +29921,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Protocolo futuro</t>
+          <t>Divergencias</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -29509,9 +29946,9 @@
           <t>0 pronto</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>DIVIDA</t>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>7 pontos</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -29595,17 +30032,17 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Protagonistas</t>
+          <t>Fontes divergentes</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Corpo real + corpo da Vila + premissa</t>
+          <t>Nome, pasta, app e lore precisam bater</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Completar vinculo e transformar lore em mecanica/mesa.</t>
+          <t>Resolver vermelhos e aceitar aliases amarelos.</t>
         </is>
       </c>
     </row>
@@ -29617,37 +30054,59 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
+          <t>Protagonistas</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Corpo real + corpo da Vila + premissa</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Completar vinculo e transformar lore em mecanica/mesa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
           <t>Mundo/Biomas</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Usar o MUN como fonte de mapa</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Separar por bioma, risco, faccao e conteudo pendente.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Mesa atual</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Baseline confiavel</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Nao mexer no app ate a planilha virar fonte clara.</t>
         </is>
@@ -29712,12 +30171,12 @@
     <hyperlink ref="A12" location="'Faccoes'!A1" display="Faccoes"/>
     <hyperlink ref="C12" location="'Conteudo_Futuro'!A1" display="Tema personagens"/>
     <hyperlink ref="E12" location="'Conteudo_Futuro'!A1" display="Topdown animado"/>
-    <hyperlink ref="G12" location="'Backlog'!A1" display="Protocolo futuro"/>
+    <hyperlink ref="G12" location="'Divergencias'!A1" display="Divergencias"/>
     <hyperlink ref="I12" location="'Core_vs_Pack'!A1" display="Release core"/>
     <hyperlink ref="A13" location="'Faccoes'!A1" display="6 grupos"/>
     <hyperlink ref="C13" location="'Conteudo_Futuro'!A1" display="5 vazios"/>
     <hyperlink ref="E13" location="'Conteudo_Futuro'!A1" display="0 pronto"/>
-    <hyperlink ref="G13" location="'Backlog'!A1" display="DIVIDA"/>
+    <hyperlink ref="G13" location="'Divergencias'!A1" display="7 pontos"/>
     <hyperlink ref="I13" location="'Core_vs_Pack'!A1" display="328.8 MiB"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implement canonical character stages and packaged validation
</commit_message>
<xml_diff>
--- a/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
+++ b/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
@@ -524,8 +524,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ControleRegrasTable" displayName="ControleRegrasTable" ref="G13:G28" headerRowCount="1">
-  <autoFilter ref="G13:G28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ControleRegrasTable" displayName="ControleRegrasTable" ref="G13:G29" headerRowCount="1">
+  <autoFilter ref="G13:G29"/>
   <tableColumns count="1">
     <tableColumn id="7" name="Regra"/>
   </tableColumns>
@@ -643,8 +643,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AppBaseChecklistTable" displayName="AppBaseChecklistTable" ref="A4:F22" headerRowCount="1">
-  <autoFilter ref="A4:F22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AppBaseChecklistTable" displayName="AppBaseChecklistTable" ref="A4:F23" headerRowCount="1">
+  <autoFilter ref="A4:F23"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Status"/>
     <tableColumn id="2" name="Area"/>
@@ -1059,7 +1059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -1442,6 +1442,13 @@
       <c r="G28" s="8" t="inlineStr">
         <is>
           <t>Combat V2 e a fonte ativa para CA, Bloqueio, Esquiva, critico, manobras, escala de mobs e simulacao; FUSHI_COMBAT_V2.md prevalece sobre regra V1 conflitante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Estagios/Fases usam uma unica ficha canonica ativa; catalogo privado do Mestre fica em snapshots nao recursivos, Jogador recebe apenas fase ativa e revision, e toda troca precisa de VFX idempotente e teste Mestre &gt; Jogador.</t>
         </is>
       </c>
     </row>
@@ -22483,7 +22490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -22703,7 +22710,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>OK tecnico</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -22713,22 +22720,22 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Efeitos e marcas canonicos</t>
+          <t>Estagios/Fases da ficha</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Origem ve Seus efeitos; alvo ve Efeitos aplicados; somente origem autorizada ou Mestre cancela; jogador nao recebe IDs internos.</t>
+          <t>Mestre cria, edita, renomeia, troca e arquiva fases; a fase ativa continua sendo a ficha canonica e jogadores recebem somente fase ativa, imagem atual e revision.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Alpha.88: Analise Cirurgica usa efeito estruturado com origem/alvo; smoke:multiplayer validou cancelamento Jogador &gt; Mestre, ACK idempotente, persistencia canonica e sanitizacao publica.</t>
+          <t>Alpha.88: smoke:stages, smoke:multiplayer, smoke:ui, smoke:release e smoke:release:deep passaram; release empacotado criou, ativou e retornou de uma fase sem vazar catalogo.</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Playtest fisico com Davi aplicando e cancelando a marca em outro jogador.</t>
+          <t>Playtest fisico com Mestre + Jogador: trocar fase, editar imagem/vida, confirmar VFX unico e retorno sem novo aceite.</t>
         </is>
       </c>
     </row>
@@ -22740,27 +22747,27 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Eventos</t>
+          <t>Ficha</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>EVE publico efemero</t>
+          <t>Efeitos e marcas canonicos</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Sorteio atual aparece aos jogadores e pode ser dispensado; backlog e ultimo roll nao reaparecem ao voltar para a mesa.</t>
+          <t>Origem ve Seus efeitos; alvo ve Efeitos aplicados; somente origem autorizada ou Mestre cancela; jogador nao recebe IDs internos.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Alpha.87 cobre transmissao depois da reconexao, descarte pelo jogador e ausencia de replay nos smokes de eventos, multiplayer e release real.</t>
+          <t>Alpha.88: Analise Cirurgica usa efeito estruturado com origem/alvo; smoke:multiplayer validou cancelamento Jogador &gt; Mestre, ACK idempotente, persistencia canonica e sanitizacao publica.</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Todo novo EVE publico precisa de teste empacotado com visao de jogador.</t>
+          <t>Playtest fisico com Davi aplicando e cancelando a marca em outro jogador.</t>
         </is>
       </c>
     </row>
@@ -22772,27 +22779,27 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Dados</t>
+          <t>Eventos</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Fila, cooldown e idempotencia</t>
+          <t>EVE publico efemero</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Rolagens rapidas nao duplicam por retry/lag.</t>
+          <t>Sorteio atual aparece aos jogadores e pode ser dispensado; backlog e ultimo roll nao reaparecem ao voltar para a mesa.</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Usuario testou e nao bugou.</t>
+          <t>Alpha.87 cobre transmissao depois da reconexao, descarte pelo jogador e ausencia de replay nos smokes de eventos, multiplayer e release real.</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Manter smoke:multiplayer.</t>
+          <t>Todo novo EVE publico precisa de teste empacotado com visao de jogador.</t>
         </is>
       </c>
     </row>
@@ -22804,27 +22811,27 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Regua</t>
+          <t>Dados</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Regua multiplayer</t>
+          <t>Fila, cooldown e idempotencia</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Linha e label aparecem sem flicker forte para Mestre e Jogador.</t>
+          <t>Rolagens rapidas nao duplicam por retry/lag.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Reforcada e testada depois do bug.</t>
+          <t>Usuario testou e nao bugou.</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Revalidar em sessao longa.</t>
+          <t>Manter smoke:multiplayer.</t>
         </is>
       </c>
     </row>
@@ -22836,27 +22843,27 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Tokens</t>
+          <t>Regua</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Controle e visual de token</t>
+          <t>Regua multiplayer</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Mestre move; jogador nao move; borda/visibilidade nao usa transparencia feia.</t>
+          <t>Linha e label aparecem sem flicker forte para Mestre e Jogador.</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Fluxo observado como responsivo.</t>
+          <t>Reforcada e testada depois do bug.</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Revalidar com 5 jogadores.</t>
+          <t>Revalidar em sessao longa.</t>
         </is>
       </c>
     </row>
@@ -22868,27 +22875,27 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Interludios</t>
+          <t>Tokens</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>MUN e mapas com thumb/topdown</t>
+          <t>Controle e visual de token</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Abrir mapa nao fica branco/preto; interludio tem thumb e fallback coerente.</t>
+          <t>Mestre move; jogador nao move; borda/visibilidade nao usa transparencia feia.</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Alpha.88: 121/121 interludios automaticos possuem fonte valida no pacote, 0 thumbs vazias; Estatuas do Litoral usa a imagem semantica do MUN; cinco ciclos empacotados e 0 falhas de rede.</t>
+          <t>Fluxo observado como responsivo.</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Revisao artistica por cena; manter a auditoria semantica antes de cada release.</t>
+          <t>Revalidar com 5 jogadores.</t>
         </is>
       </c>
     </row>
@@ -22900,27 +22907,27 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Base/MUN</t>
+          <t>Interludios</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Liberar Base/MUN e preparar mapa</t>
+          <t>MUN e mapas com thumb/topdown</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Mestre prepara sem puxar jogadores; ativar leva jogadores ao mapa correto.</t>
+          <t>Abrir mapa nao fica branco/preto; interludio tem thumb e fallback coerente.</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Alpha.84 validada no release empacotado: preparar mapa, voltar ao submapa e liberar Base passaram no smoke:release:deep.</t>
+          <t>Alpha.88: 121/121 interludios automaticos possuem fonte valida no pacote, 0 thumbs vazias; Estatuas do Litoral usa a imagem semantica do MUN; cinco ciclos empacotados e 0 falhas de rede.</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Revalidar apenas se o protocolo MUN/Base mudar.</t>
+          <t>Revisao artistica por cena; manter a auditoria semantica antes de cada release.</t>
         </is>
       </c>
     </row>
@@ -22932,27 +22939,27 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Base/MUN</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Build empacotado real</t>
+          <t>Liberar Base/MUN e preparar mapa</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>release/win-unpacked abre e smokes rodam isolados.</t>
+          <t>Mestre prepara sem puxar jogadores; ativar leva jogadores ao mapa correto.</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Alpha.87 empacotada em release/win-unpacked e instaladores; build, lint, release:assets, smoke:ui, smoke:multiplayer, smoke:release e smoke:release:deep 11/11 aprovados.</t>
+          <t>Alpha.84 validada no release empacotado: preparar mapa, voltar ao submapa e liberar Base passaram no smoke:release:deep.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Nao promover conteudo sem smoke:release e o gate especifico da area alterada.</t>
+          <t>Revalidar apenas se o protocolo MUN/Base mudar.</t>
         </is>
       </c>
     </row>
@@ -22964,59 +22971,59 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Build empacotado real</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>release/win-unpacked abre e smokes rodam isolados.</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Alpha.87 empacotada em release/win-unpacked e instaladores; build, lint, release:assets, smoke:ui, smoke:multiplayer, smoke:release e smoke:release:deep 11/11 aprovados.</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Nao promover conteudo sem smoke:release e o gate especifico da area alterada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
           <t>Livros</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Livro do Jogador e Livro do Mestre</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Jogador consulta regras publicas no Fluxo e na Mesa sem ver reencarnacao/progressao oculta; Mestre consulta escudo e compendio real; PDFs passam auditoria visual e de sigilo.</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Combat V2: 15 capitulos publicos, 18 capitulos do Mestre, PDF Jogador 23 paginas, PDF Mestre 363 paginas; auditoria visual, sigilo e bordas aprovada.</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Atualizar src/data/rulebook a cada decisao aprovada; rodar books:build, books:audit e smoke:rulebooks:release.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>FOCO</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Combate</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Combat V2 - defesa, critico e turnos</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>CA e passiva; Bloqueio usa Fortitude (0/5/10/15); Esquiva fixa usa CA atual + AGI + Reflexos como Reacao; critico dobra apenas dados; turnos mostram Principal, Curta, Movimento, Reacao e manobras.</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Alpha.88: 56 fichas Combat V2; fluxo visual ficha -&gt; Dados de Combate -&gt; dado -&gt; Resolver -&gt; confirmacao; recibo privado, impacto, marca e queda protegidos por smokes runtime, UI e multiplayer.</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Playtest fisico curto Mestre/Jogador para confirmar leitura e ritmo; manter Veyra e demais lacunas de conteudo como alerta ate revisao canonica do Mestre.</t>
         </is>
       </c>
     </row>
@@ -23028,59 +23035,59 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
+          <t>Combate</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Combat V2 - defesa, critico e turnos</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>CA e passiva; Bloqueio usa Fortitude (0/5/10/15); Esquiva fixa usa CA atual + AGI + Reflexos como Reacao; critico dobra apenas dados; turnos mostram Principal, Curta, Movimento, Reacao e manobras.</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Alpha.88: 56 fichas Combat V2; fluxo visual ficha -&gt; Dados de Combate -&gt; dado -&gt; Resolver -&gt; confirmacao; recibo privado, impacto, marca e queda protegidos por smokes runtime, UI e multiplayer.</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Playtest fisico curto Mestre/Jogador para confirmar leitura e ritmo; manter Veyra e demais lacunas de conteudo como alerta ate revisao canonica do Mestre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
           <t>Builds</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Catalogo, raridades e vinculo BUI</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>48 itens, cinco raridades, conjuntos de NPC e vinculo canonico funcionam sem alterar lore ou aceitar sobrescrita do Jogador.</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Baseline canonico aprovado por smoke:builds: 48 itens, 240 raridades e 41 conjuntos 8/8. Alpha.87 separa valor base do efetivo: editar base reaplica o total da build e remover item restaura a base sem residuo; smoke:ui e multiplayer protegem o contrato.</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Em teste real: editar a Vida base de Connor para 20, confirmar 34 com Build +14, remover a build e confirmar retorno a 20. Ajustar numeros somente com evidencia de playtest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Eventos</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Hub EVE e ciclo de vida</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Mestre ativa dois ou mais eventos, desativa cada um isoladamente e a Mesa volta ao estado-base sem apagar progresso.</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Treino Inicial e Sorteio Raridade Build passaram em build, smoke:events, smoke:training:ui, smoke:multiplayer, smoke:release e smoke:release:deep 11/11; campos privados foram removidos do payload do Jogador e a revelacao agora fecha por clique sem alterar ficha/EVE.</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Manter em teste real; todo evento novo deve seguir FUSHI_EVENT_SYSTEM_V1 e ganhar smoke proprio.</t>
         </is>
       </c>
     </row>
@@ -23092,25 +23099,57 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
+          <t>Eventos</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Hub EVE e ciclo de vida</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Mestre ativa dois ou mais eventos, desativa cada um isoladamente e a Mesa volta ao estado-base sem apagar progresso.</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Treino Inicial e Sorteio Raridade Build passaram em build, smoke:events, smoke:training:ui, smoke:multiplayer, smoke:release e smoke:release:deep 11/11; campos privados foram removidos do payload do Jogador e a revelacao agora fecha por clique sem alterar ficha/EVE.</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Manter em teste real; todo evento novo deve seguir FUSHI_EVENT_SYSTEM_V1 e ganhar smoke proprio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
           <t>Treinamento</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Circuito do Centro no Campo de Treinamento</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Mestre ativa/desativa pelo EVE ou MUN; cinco jogadores veem quests e progresso; somente Mestre ve DT e aplica Marcas, Contratempos e Segundo Sino.</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>smoke:training, smoke:training:ui e smoke:multiplayer aprovados; desativacao remove o painel em Mestre/Jogador, preserva a Marca e permite retomar.</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Teste real na proxima sessao; refinamento narrativo e habilidades continuam dependendo de aprovacao do Mestre.</t>
         </is>

</xml_diff>

<commit_message>
chore: close alpha91 rulebook refresh
</commit_message>
<xml_diff>
--- a/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
+++ b/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
@@ -2,29 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle" sheetId="1" r:id="Rb34d6f3f40ba4d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Base" sheetId="2" r:id="Rd5d1cbf8316f42fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campanha_Checklist" sheetId="3" r:id="R189d1b971525438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas_Controle" sheetId="4" r:id="R7468820385a74c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPCs_Mobs" sheetId="5" r:id="R87ae2d430e344a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Rituais" sheetId="6" r:id="R37f1892c2eb0417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biomas_Mapas" sheetId="7" r:id="Rc96134a8368642d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio_VFX" sheetId="8" r:id="R896d91e797c949b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="9" r:id="Rf55c6bbd54c542df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="10" r:id="R58b61ee621114ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="11" r:id="R3f6254925d37490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divergencias" sheetId="12" r:id="R3b47fdd91dbb4033"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core_vs_Pack" sheetId="13" r:id="Rbd3e1943f7b64153"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUN_Assets" sheetId="14" r:id="Ra00633e989694bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peso_Assets" sheetId="15" r:id="Rfd90d8ab996743d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist_Teste" sheetId="16" r:id="Rbef9b707970244e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens_Campanha" sheetId="17" r:id="R0807bcdac31940ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC_Mecanicas" sheetId="18" r:id="R56c7036a91754057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas" sheetId="19" r:id="Raea1db5902e44f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Fases" sheetId="20" r:id="R5d1b8e13e1764f34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faccoes" sheetId="21" r:id="R8f646d1ba6da41c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mundo_Biomas" sheetId="22" r:id="Rfd64d44fd42b420c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteudo_Futuro" sheetId="23" r:id="R919bced9a4f2483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle" sheetId="1" r:id="R58a2119c761e4235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Base" sheetId="2" r:id="Red6cffb8da3d4279"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campanha_Checklist" sheetId="3" r:id="R15b24491e4104d60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas_Controle" sheetId="4" r:id="Rc9e73734459045c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPCs_Mobs" sheetId="5" r:id="R893fe97797be4bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Rituais" sheetId="6" r:id="R60e98b7f71ee4700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biomas_Mapas" sheetId="7" r:id="R45b55c9698924254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio_VFX" sheetId="8" r:id="Rd157a6646fec4ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="9" r:id="Rdc71ff5019954454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="10" r:id="Re8513a79b845476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="11" r:id="Rd679f8db85f6424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divergencias" sheetId="12" r:id="R07c9ecfa66c64e6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core_vs_Pack" sheetId="13" r:id="Ra2ae65209c0e4241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUN_Assets" sheetId="14" r:id="R38d78982a02b43ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peso_Assets" sheetId="15" r:id="R0b80300a22d2423b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist_Teste" sheetId="16" r:id="R9ca3b4442e864bf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens_Campanha" sheetId="17" r:id="R5447a86c28034918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC_Mecanicas" sheetId="18" r:id="R4cf3f64ea6504687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas" sheetId="19" r:id="Rb131b8b91eed4ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Fases" sheetId="20" r:id="R2ca8062185804edb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faccoes" sheetId="21" r:id="Re977664bb8ab4c3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mundo_Biomas" sheetId="22" r:id="R792eab5ec442457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteudo_Futuro" sheetId="23" r:id="R533527ea84b3477e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -138,7 +138,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="31">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -215,6 +215,81 @@
         <x:fgColor rgb="FFF7C1C1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE7A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7C1C1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE7A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7C1C1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE7A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7C1C1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE7A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7C1C1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE7A8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7C1C1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="4">
     <x:border/>
@@ -264,7 +339,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="92">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -404,6 +479,133 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="20" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="20" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="23" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="24" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="26" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="26" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="27" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="27" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="28" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="29" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="29" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="30" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="30" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="28" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="28" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1279,7 +1481,7 @@
         </x:is>
       </x:c>
       <x:c r="D14" s="36" t="str">
-        <x:v>Alpha.90 promovida: mapas, recovery e Dia/Noite fechados. Livro, MSC e VFX seguem como frentes separadas.</x:v>
+        <x:v>Alpha.91 promovida: mapas, recovery, Dia/Noite e livros fechados tecnicamente. MSC e VFX seguem como frentes separadas.</x:v>
       </x:c>
       <x:c r="E14" s="8" t="inlineStr">
         <x:is>
@@ -1474,10 +1676,8 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="G23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Combat V2 e a fonte ativa para CA, Bloqueio, Esquiva, critico, manobras, escala de mobs e simulacao; a correcao canonica de 2026-07-13 tornou Esquiva fixa, mas runtime/Livros aguardam o checkmate da matematica.</x:t>
-        </x:is>
+      <x:c r="G23" s="8" t="str">
+        <x:v>Combat V2 e a fonte ativa para CA, Bloqueio, Esquiva, critico, manobras, escala de mobs e simulacao; FUSHI_COMBAT_V2.md prevalece sobre regra V1 conflitante; qualquer ajuste numerico segue aprovado pelo Mestre e playtest.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1508,11 +1708,9 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="G28" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Combat V2 e a fonte ativa para CA, Bloqueio, Esquiva, critico, manobras, escala de mobs e simulacao; FUSHI_COMBAT_V2.md prevalece sobre regra V1 conflitante.</x:t>
-        </x:is>
+    <x:row r="28" ht="54" customHeight="1">
+      <x:c r="G28" s="36" t="str">
+        <x:v>Alpha.91: livros nascem dos JSONs; contagens e paginas sao derivadas; auditoria reprova rotulos editoriais crus; release real 0.1.0-alpha.91.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1526,6 +1724,9 @@
       <x:c r="G30" s="37" t="str">
         <x:v>Alpha.90: preservar a ultima superficie decodificada; Ctrl+A nao troca estado; Relogio MUN e fonte de Dia/Noite; so Mestre edita luzes.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="31" ht="18" customHeight="1">
+      <x:c r="G31" s="37"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1560,8 +1761,8 @@
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd43afade6c34567"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf10efd0c1d384c9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re69556f1f0f44edd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R662adc429a554e0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1577,7 +1778,7 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>FUSHI App Readiness - Alpha.90</x:v>
+        <x:v>FUSHI App Readiness - Alpha.91</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="19" customHeight="1">
@@ -1639,7 +1840,7 @@
       <x:c r="B7" s="8" t="n">
         <x:v>4422.7</x:v>
       </x:c>
-      <x:c r="C7" s="39" t="str">
+      <x:c r="C7" s="85" t="str">
         <x:v>Pack atual; alvo de otimizacao</x:v>
       </x:c>
     </x:row>
@@ -1668,7 +1869,7 @@
         <x:v>349.2</x:v>
       </x:c>
       <x:c r="C9" s="7" t="str">
-        <x:v>Core alpha.90 validado</x:v>
+        <x:v>Core alpha.91 validado</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1793,12 +1994,12 @@
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="40" t="str">
-        <x:v>Gate alpha.90</x:v>
-      </x:c>
-      <x:c r="B18" s="42" t="n">
+        <x:v>Gate alpha.91</x:v>
+      </x:c>
+      <x:c r="B18" s="87" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C18" s="42" t="str">
+      <x:c r="C18" s="87" t="str">
         <x:v>12/12 smokes profundos no release real</x:v>
       </x:c>
     </x:row>
@@ -1806,11 +2007,22 @@
       <x:c r="A19" s="40" t="str">
         <x:v>Dia/Noite</x:v>
       </x:c>
-      <x:c r="B19" s="42" t="str">
+      <x:c r="B19" s="87" t="str">
         <x:v>OK tecnico</x:v>
       </x:c>
-      <x:c r="C19" s="42" t="str">
+      <x:c r="C19" s="87" t="str">
         <x:v>Mestre edita; Jogador recebe o visual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="40" t="str">
+        <x:v>Livros</x:v>
+      </x:c>
+      <x:c r="B20" s="87" t="str">
+        <x:v>OK tecnico</x:v>
+      </x:c>
+      <x:c r="C20" s="87" t="str">
+        <x:v>16/19 capitulos; PDFs 28/392; sigilo e auditoria visual aprovados</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1820,7 +2032,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3af52b1e2f284ec0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5752b32a315c4d9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2208,7 +2420,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743b760dda6b4f7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dc99cc3aa9e4b72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2578,7 +2790,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2bbc72c82d74854"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R544027cb9c32488b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2904,7 +3116,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2568b769228d4220"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd632f1c039fa423c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9498,7 +9710,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf16d7fd543bb4820"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R307854ca5e2d46b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12054,7 +12266,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2444f06047844b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14141bea2f654d6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12080,7 +12292,7 @@
     </x:row>
     <x:row r="2" ht="19" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Gate obrigatorio da alpha.90 e de qualquer build futura que toque multiplayer, ficha, combate, cena ou eventos.</x:v>
+        <x:v>Gate obrigatorio da alpha.91 e de qualquer build futura que toque multiplayer, ficha, combate, cena, livros ou eventos.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -12596,7 +12808,7 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
-      <x:c r="A20" s="45" t="str">
+      <x:c r="A20" s="89" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="B20" s="40" t="str">
@@ -12611,12 +12823,12 @@
       <x:c r="E20" s="40" t="str">
         <x:v>Smoke interludios + release real</x:v>
       </x:c>
-      <x:c r="F20" s="42" t="str">
-        <x:v>OK automatizado alpha.90</x:v>
+      <x:c r="F20" s="87" t="str">
+        <x:v>OK automatizado alpha.91</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
-      <x:c r="A21" s="45" t="str">
+      <x:c r="A21" s="89" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="B21" s="40" t="str">
@@ -12631,12 +12843,12 @@
       <x:c r="E21" s="40" t="str">
         <x:v>Smoke lighting + multiplayer + deep</x:v>
       </x:c>
-      <x:c r="F21" s="48" t="str">
-        <x:v>OK tecnico alpha.90; teste fisico recomendado</x:v>
+      <x:c r="F21" s="91" t="str">
+        <x:v>OK tecnico alpha.90; alpha.91 revalidado; teste fisico recomendado</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
-      <x:c r="A22" s="45" t="str">
+      <x:c r="A22" s="89" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="B22" s="40" t="str">
@@ -12651,12 +12863,12 @@
       <x:c r="E22" s="40" t="str">
         <x:v>12 smokes empacotados + release real</x:v>
       </x:c>
-      <x:c r="F22" s="42" t="str">
-        <x:v>OK automatizado alpha.90</x:v>
+      <x:c r="F22" s="87" t="str">
+        <x:v>OK automatizado alpha.91</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
-      <x:c r="A23" s="48" t="str">
+      <x:c r="A23" s="91" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="B23" s="40" t="str">
@@ -12671,8 +12883,48 @@
       <x:c r="E23" s="40" t="str">
         <x:v>npm audit --omit=dev + bundle:audit</x:v>
       </x:c>
-      <x:c r="F23" s="48" t="str">
+      <x:c r="F23" s="91" t="str">
         <x:v>ATENCAO - divida registrada</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="54" customHeight="1">
+      <x:c r="A24" s="89" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="B24" s="40" t="str">
+        <x:v>Livros e sigilo</x:v>
+      </x:c>
+      <x:c r="C24" s="40" t="str">
+        <x:v>Abrir o Livro do Jogador e o do Mestre no executavel e pesquisar uma regra publica.</x:v>
+      </x:c>
+      <x:c r="D24" s="40" t="str">
+        <x:v>Jogador tem somente regra publica; Mestre acessa compendio; capitulos e PDFs batem com a fonte.</x:v>
+      </x:c>
+      <x:c r="E24" s="40" t="str">
+        <x:v>books:build + books:audit + smoke:rulebooks:release</x:v>
+      </x:c>
+      <x:c r="F24" s="87" t="str">
+        <x:v>OK automatizado alpha.91</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" s="89" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="B25" s="40" t="str">
+        <x:v>Multiplayer soak</x:v>
+      </x:c>
+      <x:c r="C25" s="40" t="str">
+        <x:v>Repetir entrada, sair para Fluxo/Livro, voltar, editar ficha, rolar e reconectar em cinco instancias.</x:v>
+      </x:c>
+      <x:c r="D25" s="40" t="str">
+        <x:v>Nao volta para pending na mesma instancia; dados, ficha, EVE e privacidade permanecem consistentes.</x:v>
+      </x:c>
+      <x:c r="E25" s="40" t="str">
+        <x:v>smoke:multiplayer + smoke:multiplayer:soak</x:v>
+      </x:c>
+      <x:c r="F25" s="91" t="str">
+        <x:v>OK automatizado alpha.91; teste fisico recomendado</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12682,7 +12934,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83a8e4ff54394488"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a19763e8f1446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16198,7 +16450,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9716f0582c774bae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ca404fa13324bdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22536,7 +22788,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R306e818c55334441"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875ed12be63e4bfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23098,7 +23350,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2acae17d0c27426e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f1d7d12ce4d41a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23194,7 +23446,7 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6" s="42" t="str">
+      <x:c r="A6" s="87" t="str">
         <x:v>OK</x:v>
       </x:c>
       <x:c r="B6" s="27" t="str">
@@ -23207,7 +23459,7 @@
         <x:v>Entrar como Mestre, mapa e tokens aparecem, sem readiness preso; Ctrl+A recupera apenas a arte visual sem trocar mapa, tokens, camera ou sessao.</x:v>
       </x:c>
       <x:c r="E6" s="27" t="str">
-        <x:v>Alpha.90: smoke:ui e smoke:release aprovados; 79 amostras, 0 quadros vazios e Ctrl+A preservando mapa, tokens e sessao.</x:v>
+        <x:v>Alpha.91: smoke:ui, smoke:release e smoke:release:deep aprovados; recuperacao visual preservando mapa, tokens e sessao.</x:v>
       </x:c>
       <x:c r="F6" s="27" t="str">
         <x:v>Playtest fisico em dois PCs com troca repetida; Ctrl+A e apenas recuperacao do renderer.</x:v>
@@ -23502,7 +23754,7 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
-      <x:c r="A16" s="42" t="str">
+      <x:c r="A16" s="87" t="str">
         <x:v>OK</x:v>
       </x:c>
       <x:c r="B16" s="27" t="str">
@@ -23515,7 +23767,7 @@
         <x:v>Abrir mapa nao fica branco/preto; interludio tem thumb e fallback coerente.</x:v>
       </x:c>
       <x:c r="E16" s="27" t="str">
-        <x:v>Alpha.90: 121/121 fontes validas, 0 thumbs vazias, 0 quadros vazios nos ciclos e 0 falhas de rede.</x:v>
+        <x:v>Alpha.91: 121/121 fontes validas, 0 thumbs vazias, 0 quadros vazios nos ciclos e 0 falhas de rede.</x:v>
       </x:c>
       <x:c r="F16" s="27" t="str">
         <x:v>Revisao artistica por cena; manter auditoria semantica antes de cada release.</x:v>
@@ -23554,7 +23806,7 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
-      <x:c r="A18" s="42" t="str">
+      <x:c r="A18" s="87" t="str">
         <x:v>OK</x:v>
       </x:c>
       <x:c r="B18" s="27" t="str">
@@ -23567,42 +23819,30 @@
         <x:v>release/win-unpacked abre e os smokes rodam isolados.</x:v>
       </x:c>
       <x:c r="E18" s="27" t="str">
-        <x:v>Alpha.90: build, lint, UI, multiplayer, release, lighting, interludios, performance e deep 12/12 aprovados.</x:v>
+        <x:v>Alpha.91: build, lint, UI, multiplayer, soak 5/5, release e deep 12/12 aprovados; executavel versionado 0.1.0-alpha.91.</x:v>
       </x:c>
       <x:c r="F18" s="27" t="str">
         <x:v>Fechar o executavel oficial antes de empacotar e repetir o gate especifico da area.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">OK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B19" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Livros</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Livro do Jogador e Livro do Mestre</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D19" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Jogador consulta regras publicas no Fluxo e na Mesa sem ver reencarnacao/progressao oculta; Mestre consulta escudo e compendio real; PDFs passam auditoria visual e de sigilo.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E19" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Combat V2: 15 capitulos publicos, 18 capitulos do Mestre, PDF Jogador 23 paginas, PDF Mestre 363 paginas; auditoria visual, sigilo e bordas aprovada.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F19" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Atualizar src/data/rulebook a cada decisao aprovada; rodar books:build, books:audit e smoke:rulebooks:release.</x:t>
-        </x:is>
+    <x:row r="19" ht="54" customHeight="1">
+      <x:c r="A19" s="87" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Livros</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>Livro do Jogador e Livro do Mestre</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Fonte unica em src/data/rulebook; Jogador sem segredos; Mestre com compendio completo.</x:v>
+      </x:c>
+      <x:c r="E19" s="27" t="str">
+        <x:v>Alpha.91: 16 capitulos publicos, 19 do Mestre, PDFs 28/392, bibliografia 17; smoke e auditoria visual aprovados.</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="str">
+        <x:v>Manter books:build, books:audit e smoke:rulebooks:release a cada mudanca editorial.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -23734,7 +23974,7 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
-      <x:c r="A24" s="42" t="str">
+      <x:c r="A24" s="87" t="str">
         <x:v>OK tecnico</x:v>
       </x:c>
       <x:c r="B24" s="40" t="str">
@@ -23747,11 +23987,39 @@
         <x:v>Relogio MUN alterna Dia/Noite; Mestre controla lanterna e ate 24 pontos; Jogador ve sem controles.</x:v>
       </x:c>
       <x:c r="E24" s="40" t="str">
-        <x:v>Alpha.90: smoke:lighting isolado e dentro do deep 12/12; multiplayer, release e perf aprovados.</x:v>
+        <x:v>Alpha.90: smoke:lighting isolado e dentro do deep 12/12; alpha.91 revalidou o fluxo empacotado.</x:v>
       </x:c>
       <x:c r="F24" s="40" t="str">
         <x:v>Playtest fisico com noite, cursor, ponto fixo, Ctrl+T, OFF/ON e troca de mapa.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" s="87" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="B25" s="40" t="str">
+        <x:v>Multiplayer</x:v>
+      </x:c>
+      <x:c r="C25" s="40" t="str">
+        <x:v>Multiplayer soak</x:v>
+      </x:c>
+      <x:c r="D25" s="40" t="str">
+        <x:v>Aceite unico por instancia, ficha nos dois sentidos, ACK/idempotencia e privacidade preservados.</x:v>
+      </x:c>
+      <x:c r="E25" s="40" t="str">
+        <x:v>Alpha.91: smoke:multiplayer e soak 5/5 loops aprovados; media 1842 ms.</x:v>
+      </x:c>
+      <x:c r="F25" s="40" t="str">
+        <x:v>Revalidar fisicamente em dois computadores antes de uma sessao.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="18" customHeight="1">
+      <x:c r="A26" s="80"/>
+      <x:c r="B26" s="40"/>
+      <x:c r="C26" s="40"/>
+      <x:c r="D26" s="40"/>
+      <x:c r="E26" s="40"/>
+      <x:c r="F26" s="40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -23760,7 +24028,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4b43c6994a84ba7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51b0779d00d049c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24889,7 +25157,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02079c2e6a3741a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6253acb6c174a60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25319,7 +25587,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f17c067af8b41d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06fc73ddaea743f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25995,7 +26263,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R561441f1237241be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ea8992839d64520"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26293,7 +26561,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14ab59975332486d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re98b01a96f114881"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26573,7 +26841,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7848778f884441e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3d9f9e06bac4f96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27027,7 +27295,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf25996534c6d4ce4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e76549441646e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29920,7 +30188,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d525b10de6144cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc445922f9cef41ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30968,7 +31236,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd9e51fb5bdb48b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb39148c193e54650"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31509,7 +31777,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R465feb5a9ec74e43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ba50808049c45c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31931,7 +32199,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43c6efa87d9b4b20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ea62b6ab5624694"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32352,7 +32620,7 @@
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e917587842f451f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93ad9493b7df40a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: make tabletop night transitions immersive
</commit_message>
<xml_diff>
--- a/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
+++ b/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>349.2</v>
+        <v>349.4</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
@@ -31595,7 +31595,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>349.2 MiB</t>
+          <t>349.4 MiB</t>
         </is>
       </c>
     </row>
@@ -31819,7 +31819,7 @@
     <hyperlink ref="C13" location="'Conteudo_Futuro'!A1" display="5 vazios"/>
     <hyperlink ref="E13" location="'Conteudo_Futuro'!A1" display="0 pronto"/>
     <hyperlink ref="G13" location="'Divergencias'!A1" display="6 pontos"/>
-    <hyperlink ref="I13" location="'Core_vs_Pack'!A1" display="349.2 MiB"/>
+    <hyperlink ref="I13" location="'Core_vs_Pack'!A1" display="349.4 MiB"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat: rework tabletop music library
</commit_message>
<xml_diff>
--- a/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
+++ b/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
@@ -643,8 +643,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AppBaseChecklistTable" displayName="AppBaseChecklistTable" ref="A4:F26" headerRowCount="1">
-  <autoFilter ref="A4:F26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AppBaseChecklistTable" displayName="AppBaseChecklistTable" ref="A4:F28" headerRowCount="1">
+  <autoFilter ref="A4:F28"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Status"/>
     <tableColumn id="2" name="Area"/>
@@ -1462,7 +1462,7 @@
     <row r="31">
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Alpha.92: Cronicas da Ilha sao publicas e o Livro da Historia e exclusivo do Mestre; VFX sao apresentacoes efemeras com vfxExpiresAt, sem replay no reconnect; MSC fica bloqueado ate o teste fisico.</t>
+          <t>Alpha.92: Cronicas da Ilha sao publicas e o Livro da Historia e exclusivo do Mestre; VFX sao apresentacoes efemeras com vfxExpiresAt, sem replay no reconnect; MSC usa uma biblioteca unica, com pastas persistentes, capas opcionais e estado sanitizado no multiplayer.</t>
         </is>
       </c>
     </row>
@@ -22504,7 +22504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -23010,66 +23010,66 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>FOCO</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Livros</t>
+          <t>Dependencias</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Livro do Jogador e Livro do Mestre</t>
+          <t>Alertas npm audit</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Jogador consulta regras publicas no Fluxo e na Mesa sem ver reencarnacao/progressao oculta; Mestre consulta escudo e compendio real; PDFs passam auditoria visual e de sigilo.</t>
+          <t>Nenhuma correcao de dependencia pode regredir launcher, navegacao, Mesa ou multiplayer; alvo final e zero alerta alto aplicavel ao runtime.</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Combat V2: 16 capitulos publicos, 19 capitulos do Mestre, PDF Jogador 28 paginas, PDF Mestre 392 paginas; auditoria visual, sigilo e bordas aprovada.</t>
+          <t>01/08/2026: 0 criticas, 0 moderadas e 3 altas residuais; brace-expansion e transitivo, react-router-dom e direto.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Atualizar src/data/rulebook a cada decisao aprovada; rodar books:build, books:audit e smoke:rulebooks:release.</t>
+          <t>Testar atualizacao em branch dedicada com build, smoke:ui, smoke:multiplayer e smoke:release; nao aplicar npm audit fix automatico na build de sessao.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>OK tecnico</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Historia</t>
+          <t>Livros</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Cronica publica e Livro da Historia</t>
+          <t>Livro do Jogador e Livro do Mestre</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Jogador ve somente acontecimentos liberados; Mestre ve continuidade, segredos e lacunas; Sessao 4 permanece pendente ate log real.</t>
+          <t>Jogador consulta regras publicas no Fluxo e na Mesa sem ver reencarnacao/progressao oculta; Mestre consulta escudo e compendio real; PDFs passam auditoria visual e de sigilo.</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Alpha.92: dois JSONs separados, PDFs publicos e confidenciais auditados; smoke:history-vfx confirmou seis secoes publicas, oito do Mestre e bloqueio de termos proibidos.</t>
+          <t>Combat V2: 16 capitulos publicos, 19 capitulos do Mestre, PDF Jogador 28 paginas, PDF Mestre 392 paginas; auditoria visual, sigilo e bordas aprovada.</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Depois da proxima sessao, atualizar primeiro o log real e somente entao regenerar os dois volumes.</t>
+          <t>Atualizar src/data/rulebook a cada decisao aprovada; rodar books:build, books:audit e smoke:rulebooks:release.</t>
         </is>
       </c>
     </row>
@@ -23081,155 +23081,155 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Cronica publica e Livro da Historia</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Jogador ve somente acontecimentos liberados; Mestre ve continuidade, segredos e lacunas; Sessao 4 permanece pendente ate log real.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Alpha.92: dois JSONs separados, PDFs publicos e confidenciais auditados; smoke:history-vfx confirmou seis secoes publicas, oito do Mestre e bloqueio de termos proibidos.</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Depois da proxima sessao, atualizar primeiro o log real e somente entao regenerar os dois volumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>OK tecnico</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
           <t>VFX</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Catalogo VFX efemero</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Preview local nao vaza; broadcast do Mestre aparece uma vez para a mesa; clear/expiracao impedem replay em reconnect e troca de mapa.</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Alpha.92: catalogo declarativo com 10 presets, vfxExpiresAt obrigatorio e filtro de pulso antigo; smoke:history-vfx e gate empacotado dedicados.</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Playtest fisico de um preview, um broadcast e um reconnect; MSC continua bloqueado ate esse teste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Playtest fisico de um preview, um broadcast e um reconnect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>OK tecnico</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Biblioteca MSC de sessao</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Pastas permanecem visiveis; busca, favoritos, tocando agora, volume, play/pause/stop, criar, editar, excluir e capas opcionais sobrevivem ao fechamento; metadados chegam ao Jogador sem vazar controles do Mestre.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Alpha.92: interface visual em grade validada no release empacotado; smoke:release edita nome/capa e reabre a biblioteca; smoke:multiplayer protege custom track, previewImage e override de faixa nativa.</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Playtest fisico Mestre/Jogador de volume, troca de pasta, edicao de capa e retorno a Mesa; depois catalogar temas por cena/personagem sem mover os arquivos atuais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>FOCO</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Combate</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Combat V2 - defesa, critico e turnos</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>CA e passiva; Bloqueio usa Fortitude (0/5/10/15); Esquiva fixa usa CA atual + AGI + Reflexos como Reacao; critico dobra apenas dados; turnos mostram Principal, Curta, Movimento, Reacao e manobras.</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>Alpha.88: 56 fichas Combat V2; fluxo visual ficha -&gt; Dados de Combate -&gt; dado -&gt; Resolver -&gt; confirmacao; recibo privado, impacto, marca e queda protegidos por smokes runtime, UI e multiplayer.</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Playtest fisico curto Mestre/Jogador para confirmar leitura e ritmo; manter Veyra e demais lacunas de conteudo como alerta ate revisao canonica do Mestre.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>FOCO</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Builds</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Catalogo, raridades e vinculo BUI</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>48 itens, cinco raridades, conjuntos de NPC e vinculo canonico funcionam sem alterar lore ou aceitar sobrescrita do Jogador.</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Baseline canonico aprovado por smoke:builds: 48 itens, 240 raridades e 41 conjuntos 8/8. Alpha.87 separa valor base do efetivo: editar base reaplica o total da build e remover item restaura a base sem residuo; smoke:ui e multiplayer protegem o contrato.</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>Em teste real: editar a Vida base de Connor para 20, confirmar 34 com Build +14, remover a build e confirmar retorno a 20. Ajustar numeros somente com evidencia de playtest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Eventos</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Hub EVE e ciclo de vida</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Mestre ativa dois ou mais eventos, desativa cada um isoladamente e a Mesa volta ao estado-base sem apagar progresso.</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Treino Inicial e Sorteio Raridade Build passaram em build, smoke:events, smoke:training:ui, smoke:multiplayer, smoke:release e smoke:release:deep 11/11; campos privados foram removidos do payload do Jogador e a revelacao agora fecha por clique sem alterar ficha/EVE.</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Manter em teste real; todo evento novo deve seguir FUSHI_EVENT_SYSTEM_V1 e ganhar smoke proprio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>OK tecnico</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Mesa</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Dia/Noite e iluminacao</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Relogio MUN alterna Dia/Noite; Mestre controla pontos e lanterna; Jogador ve o resultado sem controles; estado persiste por troca de mapa e reconexao.</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Alpha.90: smoke:lighting isolado e dentro de smoke:release:deep; 12/12 deep, smoke:multiplayer, smoke:release e perf:release aprovados; limite de 24 luzes por cena.</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Playtest fisico Mestre/Jogador com noite, cursor, ponto fixo, Ctrl+T, OFF/ON e troca de mapa.</t>
         </is>
       </c>
     </row>
@@ -23241,25 +23241,89 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
+          <t>Eventos</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Hub EVE e ciclo de vida</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Mestre ativa dois ou mais eventos, desativa cada um isoladamente e a Mesa volta ao estado-base sem apagar progresso.</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Treino Inicial e Sorteio Raridade Build passaram em build, smoke:events, smoke:training:ui, smoke:multiplayer, smoke:release e smoke:release:deep 11/11; campos privados foram removidos do payload do Jogador e a revelacao agora fecha por clique sem alterar ficha/EVE.</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Manter em teste real; todo evento novo deve seguir FUSHI_EVENT_SYSTEM_V1 e ganhar smoke proprio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>OK tecnico</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Dia/Noite e iluminacao</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Relogio MUN alterna Dia/Noite; Mestre controla pontos e lanterna; Jogador ve o resultado sem controles; estado persiste por troca de mapa e reconexao.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Alpha.90: smoke:lighting isolado e dentro de smoke:release:deep; 12/12 deep, smoke:multiplayer, smoke:release e perf:release aprovados; limite de 24 luzes por cena.</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Playtest fisico Mestre/Jogador com noite, cursor, ponto fixo, Ctrl+T, OFF/ON e troca de mapa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
           <t>Treinamento</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Circuito do Centro no Campo de Treinamento</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>Mestre ativa/desativa pelo EVE ou MUN; cinco jogadores veem quests e progresso; somente Mestre ve DT e aplica Marcas, Contratempos e Segundo Sino.</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>smoke:training, smoke:training:ui e smoke:multiplayer aprovados; desativacao remove o painel em Mestre/Jogador, preserva a Marca e permite retomar.</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Teste real na proxima sessao; refinamento narrativo e habilidades continuam dependendo de aprovacao do Mestre.</t>
         </is>
@@ -25993,7 +26057,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Preencher depois do protocolo de pack/audio.</t>
+          <t>Usar a biblioteca MSC ja estabilizada para catalogar por cena, bioma, personagem, combate, tensao, descanso, boss e interludio; nao baixar mais assets antes dessa curadoria.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: harden tabletop rendering and visual browsers
</commit_message>
<xml_diff>
--- a/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
+++ b/06_TOOLS/fushi-tabletop/docs/planejamento/FUSHI_App_Readiness_Alpha84.xlsx
@@ -2,29 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle" sheetId="1" r:id="R8c97f4f42d6848ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Base" sheetId="2" r:id="R190694e9ba31403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campanha_Checklist" sheetId="3" r:id="R4f1209d4accc4a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas_Controle" sheetId="4" r:id="R3ffe7627d42d4dbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPCs_Mobs" sheetId="5" r:id="Rcab0e9c3cd2f4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Rituais" sheetId="6" r:id="Rc0dce3dfdf4d4a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biomas_Mapas" sheetId="7" r:id="Rdb82a1c5a50340b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio_VFX" sheetId="8" r:id="Rc39683db6853413d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="9" r:id="R04dbdc13bd994b5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="10" r:id="Ref169e775cfd4fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="11" r:id="Rc398832d7cb741f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divergencias" sheetId="12" r:id="R9e0c544915ec40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core_vs_Pack" sheetId="13" r:id="R4792de19bd9844b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUN_Assets" sheetId="14" r:id="R2ad7c5fdec6d4d79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peso_Assets" sheetId="15" r:id="Rc461071add5c445a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist_Teste" sheetId="16" r:id="R4c1af7530cb2484f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens_Campanha" sheetId="17" r:id="Rb37f5b2402534614"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC_Mecanicas" sheetId="18" r:id="R067fa5c1be634bd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas" sheetId="19" r:id="Rae309086ee0741bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Fases" sheetId="20" r:id="R9c96fbf15f724c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faccoes" sheetId="21" r:id="Rd61546b555914734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mundo_Biomas" sheetId="22" r:id="R8d1c995c557f4c25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteudo_Futuro" sheetId="23" r:id="Rbe51ed96b30f496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controle" sheetId="1" r:id="Rf1f6ff680012406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App_Base" sheetId="2" r:id="Rd30c8f37080641ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campanha_Checklist" sheetId="3" r:id="R818dc156d25f4765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas_Controle" sheetId="4" r:id="R1eb345a0b4f1493d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPCs_Mobs" sheetId="5" r:id="Ra5376695aa8849e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Rituais" sheetId="6" r:id="R2562a07a13ec4a91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biomas_Mapas" sheetId="7" r:id="Rd39f9b188d2d48f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio_VFX" sheetId="8" r:id="R1464275ea6564dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="9" r:id="R86b35289ad02429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="10" r:id="R04c33f35425c4698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="11" r:id="R390580daa38849b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divergencias" sheetId="12" r:id="Rebcad0e6b98f4bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core_vs_Pack" sheetId="13" r:id="R9a18642bb80c4b08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUN_Assets" sheetId="14" r:id="R2875ce9fa7b643f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peso_Assets" sheetId="15" r:id="R3d8ec56f5d9c40c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist_Teste" sheetId="16" r:id="R6f96dc89212648f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personagens_Campanha" sheetId="17" r:id="R5599e01aafad42a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPC_Mecanicas" sheetId="18" r:id="R16b90056548642b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protagonistas" sheetId="19" r:id="R8779967d7e774282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bosses_Fases" sheetId="20" r:id="R5a0fc6cb6f804602"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faccoes" sheetId="21" r:id="R4d5377a754a8434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mundo_Biomas" sheetId="22" r:id="R9f40bc1c76c84036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteudo_Futuro" sheetId="23" r:id="Rb79af457a4b74a80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35,7 +35,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="16">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -108,8 +108,31 @@
       <x:sz val="14"/>
       <x:color rgb="FF7F1D1D"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1D2624"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF135D36"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1D2624"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF8B1E1E"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -156,6 +179,56 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6C7C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6C7C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEAD6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7FAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6C7C7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -191,7 +264,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -240,6 +313,155 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="19" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1371,6 +1593,11 @@
         <x:v>Alpha.92: Cronicas da Ilha sao publicas e o Livro da Historia e exclusivo do Mestre; VFX sao apresentacoes efemeras com vfxExpiresAt, sem replay no reconnect; MSC usa uma biblioteca unica, com pastas persistentes, capas opcionais e estado sanitizado no multiplayer; Mapas/interludios, Escudo, OBJ, NPC, BUI, EVE e VFX compartilham o mesmo navegador visual, enquanto visualThumbnails permanece privado no workspace do Mestre.</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="92" customHeight="1">
+      <x:c r="G32" s="25" t="str">
+        <x:v>Alpha.92 estabilidade 08/08: tela branca usa detector por blocos e recuperacao real do renderer; navegadores visuais usam arvore recolhida, scroll independente, Pasta+ funcional, menu de contexto, arraste para ordenar e seletores neutros. A rodada nao altera lore, protocolo multiplayer nem a regra de movimento de tokens.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A4:B4"/>
@@ -1404,8 +1631,8 @@
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Readb8e65f8f84eca"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40f5d2672cbb434e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R952780ffe3d74ac5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94dd44db5d1846e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1425,10 +1652,8 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="19" customHeight="1">
-      <x:c r="A2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fonte unica de verdade para preservar a mesa estavel e planejar conteudo.</x:t>
-        </x:is>
+      <x:c r="A2" s="2" t="str">
+        <x:v>Fonte unica de verdade para preservar a mesa estavel e planejar conteudo. Atualizado em 2026-08-08.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1641,6 +1866,39 @@
         <x:is>
           <x:t xml:space="preserve">Conteudo futuro</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="20" t="str">
+        <x:v>Gate release deep</x:v>
+      </x:c>
+      <x:c r="B18" s="60" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>12/12 no release real em 08/08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="20" t="str">
+        <x:v>Recuperacao branca</x:v>
+      </x:c>
+      <x:c r="B19" s="60" t="str">
+        <x:v>OK tecnico</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="str">
+        <x:v>Detector 6x6 + reload real</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="20" t="str">
+        <x:v>Navegadores visuais</x:v>
+      </x:c>
+      <x:c r="B20" s="60" t="str">
+        <x:v>OK tecnico</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str">
+        <x:v>Arvore, drag e scroll validados</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1650,7 +1908,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R372fff285eac43ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ba97b6fb1b34c47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2038,7 +2296,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd94fd21c309143f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61e79699996a41f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2408,7 +2666,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4e5fdb77aea47ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3fbff24187243c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2734,7 +2992,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfa22e09997f416c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfde4dc53b0b4545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9328,7 +9586,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ad72a416008474a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1baff79f88f48c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11884,7 +12142,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc47387e5d3ec4247"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbada3cc012d4c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12425,23 +12683,63 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="69" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="B20" t="str">
+      <x:c r="B20" s="65" t="str">
         <x:v>Bibliotecas visuais e thumbnails</x:v>
       </x:c>
-      <x:c r="C20" t="str">
+      <x:c r="C20" s="65" t="str">
         <x:v>Abrir MAP, Escudo, OBJ, NPC, BUI, EVE e VFX; trocar categorias; no EVE enviar capa, fechar/reabrir e remover.</x:v>
       </x:c>
-      <x:c r="D20" t="str">
+      <x:c r="D20" s="65" t="str">
         <x:v>Cada hub preserva a logica anterior; a capa persiste no Mestre; controles e metadata privados nao vazam ao Jogador.</x:v>
       </x:c>
-      <x:c r="E20" t="str">
+      <x:c r="E20" s="65" t="str">
         <x:v>Smoke UI + multiplayer + release deep</x:v>
       </x:c>
-      <x:c r="F20" t="str">
+      <x:c r="F20" s="60" t="str">
+        <x:v>OK automatizado alpha.92; teste fisico recomendado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="66" customHeight="1">
+      <x:c r="A21" s="69" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="B21" s="65" t="str">
+        <x:v>Recuperacao real da mesa branca</x:v>
+      </x:c>
+      <x:c r="C21" s="65" t="str">
+        <x:v>Forcar a superficie central branca, aguardar a sonda confirmar blocos vazios e pressionar Ctrl+A.</x:v>
+      </x:c>
+      <x:c r="D21" s="65" t="str">
+        <x:v>Nao exibe sucesso antecipado; recarrega o renderer, reconecta o teste e preserva mapa, tokens e sessao.</x:v>
+      </x:c>
+      <x:c r="E21" s="65" t="str">
+        <x:v>Smoke release deep + Electron</x:v>
+      </x:c>
+      <x:c r="F21" s="60" t="str">
+        <x:v>OK automatizado alpha.92; teste fisico recomendado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="78" customHeight="1">
+      <x:c r="A22" s="69" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="B22" s="65" t="str">
+        <x:v>Pastas e navegadores visuais</x:v>
+      </x:c>
+      <x:c r="C22" s="65" t="str">
+        <x:v>Abrir MAP/MSC/NPC; expandir MUN, recolher, criar pasta, renomear pelo contexto, arrastar para reordenar e rolar lateral/conteudo separadamente.</x:v>
+      </x:c>
+      <x:c r="D22" s="65" t="str">
+        <x:v>Filhos so aparecem com o pai aberto; ordem persiste; Pasta+ funciona; os dois scrolls nao se arrastam juntos e nenhuma acao recarrega a mesa.</x:v>
+      </x:c>
+      <x:c r="E22" s="65" t="str">
+        <x:v>Smoke UI + release deep</x:v>
+      </x:c>
+      <x:c r="F22" s="60" t="str">
         <x:v>OK automatizado alpha.92; teste fisico recomendado</x:v>
       </x:c>
     </x:row>
@@ -12452,7 +12750,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07ed89c1afac4e42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd536dc3abca54979"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15968,7 +16266,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05102001b25e4dab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0716c53e1a54c16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22306,7 +22604,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R423b39b32ae54e31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fccf17a0d8d4f09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22868,7 +23166,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcabdb5a0eb284a25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539d5e6eca0449d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22963,36 +23261,32 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="7" t="inlineStr">
+    <x:row r="6" ht="78" customHeight="1">
+      <x:c r="A6" s="61" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">OK</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="8" t="inlineStr">
+      <x:c r="B6" s="62" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Mesa</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="8" t="inlineStr">
+      <x:c r="C6" s="62" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Mesa Mestre carrega</x:t>
         </x:is>
       </x:c>
-      <x:c r="D6" s="8" t="inlineStr">
+      <x:c r="D6" s="62" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Entrar como Mestre, mapa e tokens aparecem, sem readiness preso; Ctrl+A recupera apenas a arte visual sem trocar mapa, tokens, camera ou sessao.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Alpha.90: smoke:ui e smoke:release aprovados; smoke:release:deep mediu 79 amostras, 0 quadros vazios, 11 quadros stale durante a preparacao e confirmou Ctrl+A sem trocar mapa, tokens ou sessao.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Playtest fisico em dois PCs com troca repetida de mapas; usar Ctrl+A apenas como recuperacao de renderer se uma superficie ficar branca.</x:t>
-        </x:is>
+      <x:c r="E6" s="62" t="str">
+        <x:v>Alpha.92 em 08/08: smoke:release:deep passou 12/12. A sonda forcou uma superficie 100% branca, o detector 6x6 confirmou blankTileRatio 1, o renderer recarregou de verdade e mapa, tokens e sessao foram restaurados sem falso positivo.</x:v>
+      </x:c>
+      <x:c r="F6" s="62" t="str">
+        <x:v>Playtest fisico em dois PCs com troca repetida de mapas. Ctrl+A e contingencia; o fluxo normal deve permanecer estavel sem uso do atalho.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -23347,34 +23641,32 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="7" t="inlineStr">
+    <x:row r="18" ht="70" customHeight="1">
+      <x:c r="A18" s="61" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">OK</x:t>
         </x:is>
       </x:c>
-      <x:c r="B18" s="8" t="inlineStr">
+      <x:c r="B18" s="62" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Release</x:t>
         </x:is>
       </x:c>
-      <x:c r="C18" s="8" t="inlineStr">
+      <x:c r="C18" s="62" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Build empacotado real</x:t>
         </x:is>
       </x:c>
-      <x:c r="D18" s="8" t="inlineStr">
+      <x:c r="D18" s="62" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">release/win-unpacked abre e smokes rodam isolados.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E18" s="8" t="str">
-        <x:v>Alpha.92 empacotada novamente em 02/08/2026: build e instalador passaram; smoke:release passou em execucao isolada; release:assets confirmou 349,4 MB core, 50 audios e nenhuma copia publica no ASAR; smoke:release:deep 12/12 passou.</x:v>
-      </x:c>
-      <x:c r="F18" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Nao promover conteudo sem fechar o executavel oficial, rodar smoke:release e o gate especifico da area alterada.</x:t>
-        </x:is>
+      <x:c r="E18" s="62" t="str">
+        <x:v>Alpha.92 empacotada novamente em 08/08/2026. Lint, build, smoke:ui, smoke:multiplayer, smoke:release e smoke:release:deep 12/12 passaram; instaladores offline e web foram regenerados.</x:v>
+      </x:c>
+      <x:c r="F18" s="62" t="str">
+        <x:v>Manter fechamento escopado do executavel, smoke:release e gate profundo antes de promover qualquer mudanca estrutural.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -23697,24 +23989,24 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" t="str">
+    <x:row r="29" ht="132" customHeight="1">
+      <x:c r="A29" s="63" t="str">
         <x:v>OK tecnico</x:v>
       </x:c>
-      <x:c r="B29" t="str">
+      <x:c r="B29" s="63" t="str">
         <x:v>Interface</x:v>
       </x:c>
-      <x:c r="C29" t="str">
+      <x:c r="C29" s="63" t="str">
         <x:v>Bibliotecas visuais unificadas</x:v>
       </x:c>
-      <x:c r="D29" t="str">
+      <x:c r="D29" s="63" t="str">
         <x:v>Mapas/interludios, Escudo, OBJ, NPC, BUI, EVE e VFX usam busca, categorias persistentes a esquerda e cards a direita, preservando controles, dados e permissoes de cada hub.</x:v>
       </x:c>
-      <x:c r="E29" t="str">
-        <x:v>Alpha.92: smoke:ui abriu os sete hubs no release e validou upload PNG/JPG/WebP persistente no EVE com reabertura e remocao; thumbnails privadas nao entram no payload do Jogador.</x:v>
-      </x:c>
-      <x:c r="F29" t="str">
-        <x:v>Playtest fisico: alternar pastas, editar uma capa e confirmar que Mestre/Jogador veem apenas o que devem.</x:v>
+      <x:c r="E29" s="63" t="str">
+        <x:v>Alpha.92 em 08/08: MAP/MSC/NPC usam arvore recolhida real, subpastas por expansao, scroll lateral independente, Pasta+ funcional, menu de contexto e reordenacao por arraste. BUI inicia sem ficha escolhida; BUF, TURN, NET e MUN mantiveram a logica com hierarquia visual compacta.</x:v>
+      </x:c>
+      <x:c r="F29" s="63" t="str">
+        <x:v>Playtest fisico: expandir/recolher MUN, arrastar duas pastas, criar/renomear pasta e confirmar que selecionar hubs nao dispara novo carregamento da mesa.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23724,7 +24016,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R893721ea32c445c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15ab19fa5e73489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24853,7 +25145,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R598e69f3e77c4313"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf13ae78fae364ed8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25283,7 +25575,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a49ca3bb214c79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24512572938b47bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25959,7 +26251,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf63ac40b6ad645c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e930359dfb84c89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26257,7 +26549,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e06390fdbde4143"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15d5e25145034042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26537,7 +26829,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R140c61e72ad9447a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R731e33a80d3f428c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26991,7 +27283,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b13ce6b880943aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3e1720e84cb4b95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29884,7 +30176,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d7c8e222d7d4a7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72096fe08feb446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30932,7 +31224,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b548beddbe4fa2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18e5d02a6c524d8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31473,7 +31765,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46a505829cea4221"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb35a0f285f0f4e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31895,7 +32187,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdceb0eb510754711"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20388c088abb4ffc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32316,7 +32608,7 @@
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R723e0acd02044274"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc0dae9a983b4435"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>